<commit_message>
data: forex rates 2026-04-28 09:15 IST
</commit_message>
<xml_diff>
--- a/data/2026/forex_rates_2026-04-28.xlsx
+++ b/data/2026/forex_rates_2026-04-28.xlsx
@@ -473,16 +473,16 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>SBI</t>
+          <t>HDFC</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>less than $2,500</t>
+          <t>Cash Buying</t>
         </is>
       </c>
       <c r="C2" s="2" t="n">
-        <v>93.39</v>
+        <v>94.23999999999999</v>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
@@ -498,7 +498,7 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>$2,500 to less than $5,000</t>
+          <t>less than $2,500</t>
         </is>
       </c>
       <c r="C3" s="3" t="n">
@@ -518,11 +518,11 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>$5,000 to less than $25,000</t>
+          <t>$2,500 to less than $5,000</t>
         </is>
       </c>
       <c r="C4" s="2" t="n">
-        <v>93.51000000000001</v>
+        <v>93.39</v>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
@@ -538,11 +538,11 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>$25,000 to less than $100,000</t>
+          <t>$5,000 to less than $25,000</t>
         </is>
       </c>
       <c r="C5" s="3" t="n">
-        <v>93.62</v>
+        <v>93.51000000000001</v>
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
@@ -553,16 +553,16 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>HDFC</t>
+          <t>SBI</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Cash Buying</t>
+          <t>$25,000 to less than $100,000</t>
         </is>
       </c>
       <c r="C6" s="2" t="n">
-        <v>94.23999999999999</v>
+        <v>93.62</v>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>

</xml_diff>